<commit_message>
vault backup: 2026-08-11 17:43:31
</commit_message>
<xml_diff>
--- a/ContabilidadeFinanceira/Treinos/Ex8_EditoraFarol.xlsx
+++ b/ContabilidadeFinanceira/Treinos/Ex8_EditoraFarol.xlsx
@@ -1354,7 +1354,7 @@
         <v/>
       </c>
       <c r="D31" s="11">
-        <f>IF(C31=0,"✔ fecha","✗")</f>
+        <f>IF(COUNT(C5:C26)=0,"",IF(C31=0,"✔ fecha","✗"))</f>
         <v/>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
         <v/>
       </c>
       <c r="D41" s="11">
-        <f>IF(C41=0,"✔ bate","✗")</f>
+        <f>IF(OR(COUNT(C34:C38)=0,COUNT(C5:C26)=0),"",IF(C41=0,"✔ bate","✗"))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-08-11 17:48:37
</commit_message>
<xml_diff>
--- a/ContabilidadeFinanceira/Treinos/Ex8_EditoraFarol.xlsx
+++ b/ContabilidadeFinanceira/Treinos/Ex8_EditoraFarol.xlsx
@@ -1354,7 +1354,7 @@
         <v/>
       </c>
       <c r="D31" s="11">
-        <f>IF(COUNT(C5:C26)=0,"",IF(C31=0,"✔ fecha","✗"))</f>
+        <f>IF(AND(C14=0,C19=0,C26=0),"",IF(C31=0,"✔ fecha","✗"))</f>
         <v/>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
         <v/>
       </c>
       <c r="D41" s="11">
-        <f>IF(OR(COUNT(C34:C38)=0,COUNT(C5:C26)=0),"",IF(C41=0,"✔ bate","✗"))</f>
+        <f>IF(AND(C14=0,C39=0),"",IF(C41=0,"✔ bate","✗"))</f>
         <v/>
       </c>
     </row>

</xml_diff>